<commit_message>
final changes for evaluation
</commit_message>
<xml_diff>
--- a/src/evaluation/data/processed/RES_accessibility_based_model.xlsx
+++ b/src/evaluation/data/processed/RES_accessibility_based_model.xlsx
@@ -472,22 +472,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>12.366</v>
+        <v>15.188</v>
       </c>
       <c r="C2" t="n">
         <v>12.08</v>
       </c>
       <c r="D2" t="n">
-        <v>15.662</v>
+        <v>26.57</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>0.5932565087494661</v>
       </c>
       <c r="F2" t="n">
-        <v>0.2719449225473322</v>
+        <v>0.3434782608695652</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>0.9311967068509257</v>
       </c>
     </row>
     <row r="3">
@@ -497,22 +497,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>14.74</v>
+        <v>16.23</v>
       </c>
       <c r="C3" t="n">
-        <v>14.57</v>
+        <v>18.12</v>
       </c>
       <c r="D3" t="n">
-        <v>17.74</v>
+        <v>20.236</v>
       </c>
       <c r="E3" t="n">
-        <v>0.346468184471687</v>
+        <v>0.8156209987195902</v>
       </c>
       <c r="F3" t="n">
-        <v>0.4862306368330465</v>
+        <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1826652601969056</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -531,13 +531,13 @@
         <v>23.792</v>
       </c>
       <c r="E4" t="n">
-        <v>0.006129597197898138</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>0.7146624472573837</v>
+        <v>0.522787415466039</v>
       </c>
     </row>
     <row r="5">
@@ -547,7 +547,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>17.072</v>
+        <v>17.094</v>
       </c>
       <c r="C5" t="n">
         <v>15.68</v>
@@ -556,10 +556,10 @@
         <v>27.038</v>
       </c>
       <c r="E5" t="n">
-        <v>0.6868067717454756</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>0.5817555938037866</v>
+        <v>0.734782608695652</v>
       </c>
       <c r="G5" t="n">
         <v>1</v>
@@ -572,22 +572,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>19.218</v>
+        <v>15.014</v>
       </c>
       <c r="C6" t="n">
-        <v>20.54</v>
+        <v>14.19</v>
       </c>
       <c r="D6" t="n">
-        <v>25.286</v>
+        <v>20.45</v>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>0.5561246265471615</v>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>0.5728260869565216</v>
       </c>
       <c r="G6" t="n">
-        <v>0.8459915611814347</v>
+        <v>0.03146133490149936</v>
       </c>
     </row>
     <row r="7">
@@ -597,22 +597,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>12.426</v>
+        <v>13.652</v>
       </c>
       <c r="C7" t="n">
-        <v>13.41</v>
+        <v>14.45</v>
       </c>
       <c r="D7" t="n">
-        <v>19.308</v>
+        <v>20.294</v>
       </c>
       <c r="E7" t="n">
-        <v>0.008756567425568733</v>
+        <v>0.2654716175842931</v>
       </c>
       <c r="F7" t="n">
-        <v>0.3864027538726335</v>
+        <v>0.601086956521739</v>
       </c>
       <c r="G7" t="n">
-        <v>0.3204992967651195</v>
+        <v>0.008526903851807745</v>
       </c>
     </row>
   </sheetData>

</xml_diff>